<commit_message>
run at xclude 0.8
</commit_message>
<xml_diff>
--- a/files/STable4.xlsx
+++ b/files/STable4.xlsx
@@ -6,13 +6,13 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t xml:space="preserve">
 </t>
@@ -106,6 +106,9 @@
   <si>
     <t xml:space="preserve">sdyp_hrv
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;0.9</t>
   </si>
   <si>
     <t xml:space="preserve">wl_mtr
@@ -732,28 +735,28 @@
         <v>24</v>
       </c>
       <c r="AP1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AQ1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AR1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AS1" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="AT1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AU1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AV1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="AW1" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" ht="NA" customHeight="1">
@@ -1038,8 +1041,8 @@
       <c r="AR3" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="AS3" s="9" t="s">
-        <v>15</v>
+      <c r="AS3" s="9" t="n">
+        <v>0.4</v>
       </c>
       <c r="AT3" s="9" t="s">
         <v>11</v>
@@ -1059,49 +1062,49 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F4" s="10" t="n">
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
       <c r="G4" s="10" t="n">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>0.54</v>
+        <v>0.51</v>
       </c>
       <c r="I4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="10" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="K4" s="10" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="L4" s="10" t="n">
-        <v>0.63</v>
+        <v>0.62</v>
       </c>
       <c r="M4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="N4" s="10" t="n">
-        <v>0.28</v>
+        <v>0.25</v>
       </c>
       <c r="O4" s="10" t="n">
-        <v>-0.03</v>
+        <v>0.07</v>
       </c>
       <c r="P4" s="10" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="Q4" s="10" t="s">
         <v>11</v>
@@ -1110,31 +1113,31 @@
         <v>0.16</v>
       </c>
       <c r="S4" s="10" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="T4" s="10" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="U4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="V4" s="10" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="W4" s="10" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="X4" s="10" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="Y4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z4" s="10" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="AA4" s="10" t="n">
         <v>0.34</v>
-      </c>
-      <c r="T4" s="10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="U4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="V4" s="10" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="W4" s="10" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="X4" s="10" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="Y4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z4" s="10" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="AA4" s="10" t="n">
-        <v>0.31</v>
       </c>
       <c r="AB4" s="10" t="n">
         <v>0.38</v>
@@ -1143,13 +1146,13 @@
         <v>11</v>
       </c>
       <c r="AD4" s="10" t="n">
-        <v>0.4</v>
+        <v>0.38</v>
       </c>
       <c r="AE4" s="10" t="n">
-        <v>0.22</v>
+        <v>0.28</v>
       </c>
       <c r="AF4" s="10" t="n">
-        <v>0.31</v>
+        <v>0.33</v>
       </c>
       <c r="AG4" s="10" t="s">
         <v>11</v>
@@ -1158,46 +1161,46 @@
         <v>-0.11</v>
       </c>
       <c r="AI4" s="10" t="n">
-        <v>0.33</v>
+        <v>0.31</v>
       </c>
       <c r="AJ4" s="10" t="n">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="AK4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AL4" s="10" t="n">
-        <v>0.32</v>
+        <v>0.3</v>
       </c>
       <c r="AM4" s="10" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="AN4" s="10" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="AO4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AP4" s="10" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="AQ4" s="10" t="n">
-        <v>0.27</v>
+        <v>0.22</v>
       </c>
       <c r="AR4" s="10" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="AS4" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AT4" s="10" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="AU4" s="10" t="n">
-        <v>0.26</v>
+        <v>0.29</v>
       </c>
       <c r="AV4" s="10" t="n">
-        <v>0.39</v>
+        <v>0.4</v>
       </c>
       <c r="AW4" s="10" t="s">
         <v>11</v>
@@ -1208,13 +1211,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>0.17</v>
       </c>
-      <c r="C5" s="10" t="n">
-        <v>0.15</v>
-      </c>
       <c r="D5" s="10" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>11</v>
@@ -1223,19 +1226,19 @@
         <v>0.07</v>
       </c>
       <c r="G5" s="10" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="I5" s="10" t="s">
         <v>11</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>0.07</v>
+        <v>0.08</v>
       </c>
       <c r="K5" s="10" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>0.21</v>
@@ -1244,13 +1247,13 @@
         <v>11</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>0.17</v>
       </c>
       <c r="P5" s="10" t="n">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="Q5" s="10" t="s">
         <v>11</v>
@@ -1259,10 +1262,10 @@
         <v>0.15</v>
       </c>
       <c r="S5" s="10" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="T5" s="10" t="n">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="U5" s="10" t="s">
         <v>11</v>
@@ -1271,70 +1274,70 @@
         <v>0.07</v>
       </c>
       <c r="W5" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="X5" s="10" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="Y5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z5" s="10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA5" s="10" t="n">
         <v>0.14</v>
       </c>
-      <c r="X5" s="10" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="Y5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z5" s="10" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="AA5" s="10" t="n">
+      <c r="AB5" s="10" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="AC5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD5" s="10" t="n">
         <v>0.16</v>
-      </c>
-      <c r="AB5" s="10" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AC5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD5" s="10" t="n">
-        <v>0.14</v>
       </c>
       <c r="AE5" s="10" t="n">
         <v>0.19</v>
       </c>
       <c r="AF5" s="10" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="AG5" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AH5" s="10" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="AI5" s="10" t="n">
         <v>0.16</v>
       </c>
       <c r="AJ5" s="10" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="AK5" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AL5" s="10" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="AM5" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AN5" s="10" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AO5" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP5" s="10" t="n">
         <v>0.12</v>
-      </c>
-      <c r="AM5" s="10" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AN5" s="10" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AO5" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP5" s="10" t="n">
-        <v>0.14</v>
       </c>
       <c r="AQ5" s="10" t="n">
         <v>0.14</v>
       </c>
       <c r="AR5" s="10" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="AS5" s="10" t="s">
         <v>11</v>
@@ -1343,10 +1346,10 @@
         <v>0.12</v>
       </c>
       <c r="AU5" s="10" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="AV5" s="10" t="n">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="AW5" s="10" t="s">
         <v>11</v>
@@ -1357,145 +1360,145 @@
         <v>5</v>
       </c>
       <c r="B6" s="10" t="n">
-        <v>-0.43</v>
+        <v>-0.45</v>
       </c>
       <c r="C6" s="10" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>-0.02</v>
+      </c>
+      <c r="M6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="N6" s="10" t="n">
+        <v>-0.3</v>
+      </c>
+      <c r="O6" s="10" t="n">
         <v>-0.41</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>-0.43</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>-0.15</v>
-      </c>
-      <c r="I6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="J6" s="10" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="K6" s="10" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="L6" s="10" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N6" s="10" t="n">
+      <c r="P6" s="10" t="n">
+        <v>-0.41</v>
+      </c>
+      <c r="Q6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="R6" s="10" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="S6" s="10" t="n">
         <v>-0.13</v>
       </c>
-      <c r="O6" s="10" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="P6" s="10" t="n">
-        <v>-0.52</v>
-      </c>
-      <c r="Q6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="R6" s="10" t="n">
-        <v>-0.35</v>
-      </c>
-      <c r="S6" s="10" t="n">
-        <v>-0.14</v>
-      </c>
       <c r="T6" s="10" t="n">
-        <v>-0.35</v>
+        <v>-0.46</v>
       </c>
       <c r="U6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="V6" s="10" t="n">
-        <v>0.42</v>
+        <v>0.53</v>
       </c>
       <c r="W6" s="10" t="n">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="X6" s="10" t="n">
-        <v>-0.15</v>
+        <v>-0.08</v>
       </c>
       <c r="Y6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="Z6" s="10" t="n">
-        <v>-0.04</v>
+        <v>0.1</v>
       </c>
       <c r="AA6" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.07</v>
       </c>
       <c r="AB6" s="10" t="n">
-        <v>-0.26</v>
+        <v>-0.07</v>
       </c>
       <c r="AC6" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AD6" s="10" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="AE6" s="10" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="AF6" s="10" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="AG6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH6" s="10" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="AI6" s="10" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="AJ6" s="10" t="n">
+        <v>-0.57</v>
+      </c>
+      <c r="AK6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL6" s="10" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="AM6" s="10" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="AN6" s="10" t="n">
+        <v>-0.38</v>
+      </c>
+      <c r="AO6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP6" s="10" t="n">
+        <v>-0.27</v>
+      </c>
+      <c r="AQ6" s="10" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="AR6" s="10" t="n">
+        <v>-0.36</v>
+      </c>
+      <c r="AS6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AT6" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AU6" s="10" t="n">
         <v>-0.23</v>
       </c>
-      <c r="AE6" s="10" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="AF6" s="10" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="AG6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AH6" s="10" t="n">
-        <v>-0.55</v>
-      </c>
-      <c r="AI6" s="10" t="n">
-        <v>-0.21</v>
-      </c>
-      <c r="AJ6" s="10" t="n">
-        <v>-0.55</v>
-      </c>
-      <c r="AK6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL6" s="10" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="AM6" s="10" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="AN6" s="10" t="n">
-        <v>-0.28</v>
-      </c>
-      <c r="AO6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP6" s="10" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="AQ6" s="10" t="n">
-        <v>-0.18</v>
-      </c>
-      <c r="AR6" s="10" t="n">
-        <v>-0.47</v>
-      </c>
-      <c r="AS6" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AT6" s="10" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="AU6" s="10" t="n">
-        <v>-0.25</v>
-      </c>
       <c r="AV6" s="10" t="n">
-        <v>-0.25</v>
+        <v>-0.23</v>
       </c>
       <c r="AW6" s="10" t="s">
         <v>11</v>
@@ -1506,133 +1509,133 @@
         <v>6</v>
       </c>
       <c r="B7" s="10" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.39</v>
+        <v>0.48</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.5</v>
+        <v>0.48</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="I7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="J7" s="10" t="n">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="K7" s="10" t="n">
+        <v>0.81</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="N7" s="10" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="O7" s="10" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="P7" s="10" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="Q7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="R7" s="10" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="S7" s="10" t="n">
         <v>0.82</v>
       </c>
-      <c r="L7" s="10" t="n">
-        <v>0.93</v>
-      </c>
-      <c r="M7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N7" s="10" t="n">
+      <c r="T7" s="10" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="U7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="V7" s="10" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="W7" s="10" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="X7" s="10" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="Y7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z7" s="10" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AA7" s="10" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="AB7" s="10" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="AC7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD7" s="10" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AE7" s="10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AF7" s="10" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="AG7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH7" s="10" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="AI7" s="10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AJ7" s="10" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AK7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL7" s="10" t="n">
         <v>0.59</v>
       </c>
-      <c r="O7" s="10" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="P7" s="10" t="n">
-        <v>0.59</v>
-      </c>
-      <c r="Q7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="R7" s="10" t="n">
+      <c r="AM7" s="10" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AN7" s="10" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="AO7" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP7" s="10" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="AQ7" s="10" t="n">
         <v>0.65</v>
       </c>
-      <c r="S7" s="10" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="T7" s="10" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="U7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="V7" s="10" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="W7" s="10" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="X7" s="10" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="Y7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z7" s="10" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AA7" s="10" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="AB7" s="10" t="n">
-        <v>0.76</v>
-      </c>
-      <c r="AC7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD7" s="10" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AE7" s="10" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AF7" s="10" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="AG7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AH7" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AI7" s="10" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AJ7" s="10" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AK7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL7" s="10" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AM7" s="10" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AN7" s="10" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="AO7" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP7" s="10" t="n">
-        <v>0.55</v>
-      </c>
-      <c r="AQ7" s="10" t="n">
-        <v>0.59</v>
-      </c>
       <c r="AR7" s="10" t="n">
-        <v>0.59</v>
+        <v>0.65</v>
       </c>
       <c r="AS7" s="10" t="s">
         <v>11</v>
@@ -1641,10 +1644,10 @@
         <v>0.75</v>
       </c>
       <c r="AU7" s="10" t="n">
-        <v>0.78</v>
+        <v>0.69</v>
       </c>
       <c r="AV7" s="10" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="AW7" s="10" t="s">
         <v>11</v>
@@ -1664,7 +1667,7 @@
         <v>11</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>11</v>
@@ -1712,7 +1715,7 @@
         <v>11</v>
       </c>
       <c r="U8" s="10" t="n">
-        <v>0.001</v>
+        <v>0.014</v>
       </c>
       <c r="V8" s="10" t="s">
         <v>11</v>
@@ -1735,8 +1738,8 @@
       <c r="AB8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="AC8" s="10" t="s">
-        <v>15</v>
+      <c r="AC8" s="10" t="n">
+        <v>0.3</v>
       </c>
       <c r="AD8" s="10" t="s">
         <v>11</v>
@@ -1771,8 +1774,8 @@
       <c r="AN8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="AO8" s="10" t="n">
-        <v>0.001</v>
+      <c r="AO8" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="AP8" s="10" t="s">
         <v>11</v>
@@ -1784,7 +1787,7 @@
         <v>11</v>
       </c>
       <c r="AS8" s="10" t="n">
-        <v>0.072</v>
+        <v>0.2</v>
       </c>
       <c r="AT8" s="10" t="s">
         <v>11</v>
@@ -1804,7 +1807,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="10" t="n">
-        <v>1.02</v>
+        <v>1.03</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>1.02</v>
@@ -1816,31 +1819,31 @@
         <v>11</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="I9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>0.76</v>
+        <v>0.78</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="M9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="O9" s="10" t="n">
         <v>1.02</v>
@@ -1852,7 +1855,7 @@
         <v>11</v>
       </c>
       <c r="R9" s="10" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="S9" s="10" t="n">
         <v>1</v>
@@ -1864,25 +1867,25 @@
         <v>11</v>
       </c>
       <c r="V9" s="10" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="W9" s="10" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="X9" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="Y9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="Z9" s="10" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AA9" s="10" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="AB9" s="10" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="AC9" s="10" t="s">
         <v>11</v>
@@ -1891,7 +1894,7 @@
         <v>0.97</v>
       </c>
       <c r="AE9" s="10" t="n">
-        <v>1.01</v>
+        <v>1.02</v>
       </c>
       <c r="AF9" s="10" t="n">
         <v>0.99</v>
@@ -1900,22 +1903,22 @@
         <v>11</v>
       </c>
       <c r="AH9" s="10" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="AI9" s="10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="AJ9" s="10" t="n">
         <v>1.01</v>
       </c>
-      <c r="AI9" s="10" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="AJ9" s="10" t="n">
-        <v>1</v>
-      </c>
       <c r="AK9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AL9" s="10" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="AM9" s="10" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="AN9" s="10" t="n">
         <v>1.01</v>
@@ -1924,25 +1927,25 @@
         <v>11</v>
       </c>
       <c r="AP9" s="10" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="AQ9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="AQ9" s="10" t="n">
-        <v>0.99</v>
-      </c>
       <c r="AR9" s="10" t="n">
-        <v>1</v>
+        <v>1.01</v>
       </c>
       <c r="AS9" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AT9" s="10" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="AU9" s="10" t="n">
         <v>1</v>
       </c>
       <c r="AV9" s="10" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AW9" s="10" t="s">
         <v>11</v>
@@ -1953,19 +1956,19 @@
         <v>4</v>
       </c>
       <c r="B10" s="10" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="C10" s="10" t="n">
         <v>0.05</v>
       </c>
-      <c r="C10" s="10" t="n">
+      <c r="D10" s="10" t="n">
         <v>0.06</v>
       </c>
-      <c r="D10" s="10" t="n">
-        <v>0.05</v>
-      </c>
       <c r="E10" s="10" t="s">
         <v>11</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>0.05</v>
@@ -1980,7 +1983,7 @@
         <v>0.07</v>
       </c>
       <c r="K10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="L10" s="10" t="n">
         <v>0.12</v>
@@ -1989,10 +1992,10 @@
         <v>11</v>
       </c>
       <c r="N10" s="10" t="n">
-        <v>0.07</v>
+        <v>0.06</v>
       </c>
       <c r="O10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="P10" s="10" t="n">
         <v>0.06</v>
@@ -2004,7 +2007,7 @@
         <v>0.06</v>
       </c>
       <c r="S10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.07</v>
       </c>
       <c r="T10" s="10" t="n">
         <v>0.06</v>
@@ -2013,19 +2016,19 @@
         <v>11</v>
       </c>
       <c r="V10" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="W10" s="10" t="n">
         <v>0.06</v>
       </c>
-      <c r="W10" s="10" t="n">
-        <v>0.05</v>
-      </c>
       <c r="X10" s="10" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="Y10" s="10" t="s">
         <v>11</v>
       </c>
       <c r="Z10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="AA10" s="10" t="n">
         <v>0.05</v>
@@ -2037,10 +2040,10 @@
         <v>11</v>
       </c>
       <c r="AD10" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE10" s="10" t="n">
         <v>0.06</v>
-      </c>
-      <c r="AE10" s="10" t="n">
-        <v>0.05</v>
       </c>
       <c r="AF10" s="10" t="n">
         <v>0.06</v>
@@ -2049,19 +2052,19 @@
         <v>11</v>
       </c>
       <c r="AH10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="AI10" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="AJ10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="AK10" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AL10" s="10" t="n">
-        <v>0.06</v>
+        <v>0.07</v>
       </c>
       <c r="AM10" s="10" t="n">
         <v>0.06</v>
@@ -2073,7 +2076,7 @@
         <v>11</v>
       </c>
       <c r="AP10" s="10" t="n">
-        <v>0.05</v>
+        <v>0.07</v>
       </c>
       <c r="AQ10" s="10" t="n">
         <v>0.06</v>
@@ -2085,13 +2088,13 @@
         <v>11</v>
       </c>
       <c r="AT10" s="10" t="n">
-        <v>0.07</v>
+        <v>0.06</v>
       </c>
       <c r="AU10" s="10" t="n">
         <v>0.06</v>
       </c>
       <c r="AV10" s="10" t="n">
-        <v>0.07</v>
+        <v>0.06</v>
       </c>
       <c r="AW10" s="10" t="s">
         <v>11</v>
@@ -2114,37 +2117,37 @@
         <v>11</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>0.94</v>
+        <v>0.95</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="I11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="J11" s="10" t="n">
-        <v>0.61</v>
+        <v>0.66</v>
       </c>
       <c r="K11" s="10" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="M11" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="N11" s="10" t="n">
         <v>0.88</v>
       </c>
-      <c r="L11" s="10" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="N11" s="10" t="n">
-        <v>0.89</v>
-      </c>
       <c r="O11" s="10" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="P11" s="10" t="n">
-        <v>0.89</v>
+        <v>0.88</v>
       </c>
       <c r="Q11" s="10" t="s">
         <v>11</v>
@@ -2153,46 +2156,46 @@
         <v>0.95</v>
       </c>
       <c r="S11" s="10" t="n">
-        <v>0.94</v>
+        <v>0.9</v>
       </c>
       <c r="T11" s="10" t="n">
-        <v>0.94</v>
+        <v>0.9</v>
       </c>
       <c r="U11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="V11" s="10" t="n">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="W11" s="10" t="n">
         <v>0.91</v>
       </c>
       <c r="X11" s="10" t="n">
-        <v>0.64</v>
+        <v>0.67</v>
       </c>
       <c r="Y11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="Z11" s="10" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="AA11" s="10" t="n">
-        <v>0.93</v>
+        <v>0.89</v>
       </c>
       <c r="AB11" s="10" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="AC11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AD11" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="AE11" s="10" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="AF11" s="10" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
       <c r="AG11" s="10" t="s">
         <v>11</v>
@@ -2201,22 +2204,22 @@
         <v>0.98</v>
       </c>
       <c r="AI11" s="10" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="AJ11" s="10" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="AK11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AL11" s="10" t="n">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AM11" s="10" t="n">
-        <v>0.95</v>
+        <v>0.94</v>
       </c>
       <c r="AN11" s="10" t="n">
-        <v>0.91</v>
+        <v>0.94</v>
       </c>
       <c r="AO11" s="10" t="s">
         <v>11</v>
@@ -2225,22 +2228,22 @@
         <v>0.94</v>
       </c>
       <c r="AQ11" s="10" t="n">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="AR11" s="10" t="n">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="AS11" s="10" t="s">
         <v>11</v>
       </c>
       <c r="AT11" s="10" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="AU11" s="10" t="n">
-        <v>0.92</v>
+        <v>0.89</v>
       </c>
       <c r="AV11" s="10" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="AW11" s="10" t="s">
         <v>11</v>
@@ -2251,145 +2254,145 @@
         <v>6</v>
       </c>
       <c r="B12" s="11" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>1.69</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="H12" s="11" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" s="11" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="N12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="O12" s="11" t="n">
         <v>1.29</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>0.94</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="J12" s="11" t="n">
+      <c r="P12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="Q12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="R12" s="11" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="S12" s="11" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="T12" s="11" t="n">
+        <v>1.49</v>
+      </c>
+      <c r="U12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="V12" s="11" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="W12" s="11" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="X12" s="11" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="Y12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z12" s="11" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AA12" s="11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="AB12" s="11" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="AC12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD12" s="11" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="AE12" s="11" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AF12" s="11" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AG12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH12" s="11" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AI12" s="11" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="AJ12" s="11" t="n">
+        <v>1.38</v>
+      </c>
+      <c r="AK12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AL12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="AM12" s="11" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="AN12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="AO12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AP12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="AQ12" s="11" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="AR12" s="11" t="n">
+        <v>1.43</v>
+      </c>
+      <c r="AS12" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="AT12" s="11" t="n">
         <v>1.24</v>
       </c>
-      <c r="K12" s="11" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="L12" s="11" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="M12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="N12" s="11" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="O12" s="11" t="n">
-        <v>1.24</v>
-      </c>
-      <c r="P12" s="11" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="Q12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="R12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="S12" s="11" t="n">
-        <v>1.27</v>
-      </c>
-      <c r="T12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="U12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="V12" s="11" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="W12" s="11" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="X12" s="11" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="Y12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="Z12" s="11" t="n">
-        <v>1.23</v>
-      </c>
-      <c r="AA12" s="11" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="AB12" s="11" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="AC12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AD12" s="11" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="AE12" s="11" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="AF12" s="11" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="AG12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AH12" s="11" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="AI12" s="11" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="AJ12" s="11" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="AK12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AL12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="AM12" s="11" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="AN12" s="11" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="AO12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AP12" s="11" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="AQ12" s="11" t="n">
-        <v>1.38</v>
-      </c>
-      <c r="AR12" s="11" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="AS12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="AT12" s="11" t="n">
-        <v>1.36</v>
-      </c>
       <c r="AU12" s="11" t="n">
-        <v>1.28</v>
+        <v>1.4</v>
       </c>
       <c r="AV12" s="11" t="n">
-        <v>1.36</v>
+        <v>1.4</v>
       </c>
       <c r="AW12" s="11" t="s">
         <v>11</v>

</xml_diff>